<commit_message>
one column to one method
</commit_message>
<xml_diff>
--- a/2000-2023年各省份城镇化水平.xlsx
+++ b/2000-2023年各省份城镇化水平.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13540" activeTab="2"/>
+    <workbookView windowWidth="29100" windowHeight="13520" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="面板数据" sheetId="1" r:id="rId1"/>
@@ -227,7 +227,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="132">
   <si>
     <t>id</t>
   </si>
@@ -412,7 +412,13 @@
     <t>增长率2</t>
   </si>
   <si>
+    <t>北京市</t>
+  </si>
+  <si>
     <t>87.6</t>
+  </si>
+  <si>
+    <t>天津市</t>
   </si>
   <si>
     <t>85.11</t>
@@ -421,10 +427,16 @@
     <t>85.49</t>
   </si>
   <si>
+    <t>河北省</t>
+  </si>
+  <si>
     <t>61.65</t>
   </si>
   <si>
     <t>62.77</t>
+  </si>
+  <si>
+    <t>山西省</t>
   </si>
   <si>
     <t>63.96</t>
@@ -439,10 +451,25 @@
     <t>69.58</t>
   </si>
   <si>
+    <t>辽宁省</t>
+  </si>
+  <si>
+    <t>吉林省</t>
+  </si>
+  <si>
     <t>63.73</t>
   </si>
   <si>
+    <t>黑龙江省</t>
+  </si>
+  <si>
     <t>66.2</t>
+  </si>
+  <si>
+    <t>上海市</t>
+  </si>
+  <si>
+    <t>江苏省</t>
   </si>
   <si>
     <t>74.4</t>
@@ -451,10 +478,16 @@
     <t>75.0</t>
   </si>
   <si>
+    <t>浙江省</t>
+  </si>
+  <si>
     <t>73.4</t>
   </si>
   <si>
     <t>74.2</t>
+  </si>
+  <si>
+    <t>安徽省</t>
   </si>
   <si>
     <t>60.2</t>
@@ -463,13 +496,22 @@
     <t>61.51</t>
   </si>
   <si>
+    <t>福建省</t>
+  </si>
+  <si>
     <t>70.11</t>
   </si>
   <si>
     <t>71.04</t>
   </si>
   <si>
+    <t>江西省</t>
+  </si>
+  <si>
     <t>62.07</t>
+  </si>
+  <si>
+    <t>山东省</t>
   </si>
   <si>
     <t>64.54</t>
@@ -478,10 +520,19 @@
     <t>65.53</t>
   </si>
   <si>
+    <t>河南省</t>
+  </si>
+  <si>
     <t>57.07</t>
   </si>
   <si>
+    <t>湖北省</t>
+  </si>
+  <si>
     <t>64.67</t>
+  </si>
+  <si>
+    <t>湖南省</t>
   </si>
   <si>
     <t>60.31</t>
@@ -490,10 +541,16 @@
     <t>61.16</t>
   </si>
   <si>
+    <t>广东省</t>
+  </si>
+  <si>
     <t>74.79</t>
   </si>
   <si>
     <t>55.65</t>
+  </si>
+  <si>
+    <t>海南省</t>
   </si>
   <si>
     <t>61.49</t>
@@ -502,10 +559,16 @@
     <t>62.46</t>
   </si>
   <si>
+    <t>重庆市</t>
+  </si>
+  <si>
     <t>70.96</t>
   </si>
   <si>
     <t>71.67</t>
+  </si>
+  <si>
+    <t>四川省</t>
   </si>
   <si>
     <t>58.35</t>
@@ -514,7 +577,13 @@
     <t>59.49</t>
   </si>
   <si>
+    <t>贵州省</t>
+  </si>
+  <si>
     <t>54.81</t>
+  </si>
+  <si>
+    <t>云南省</t>
   </si>
   <si>
     <t>51.72</t>
@@ -523,10 +592,19 @@
     <t>37.36</t>
   </si>
   <si>
+    <t>陕西省</t>
+  </si>
+  <si>
+    <t>甘肃省</t>
+  </si>
+  <si>
     <t>54.19</t>
   </si>
   <si>
     <t>55.49</t>
+  </si>
+  <si>
+    <t>青海省</t>
   </si>
   <si>
     <t>61.43</t>
@@ -12850,7 +12928,7 @@
     </row>
     <row r="2" spans="1:27">
       <c r="A2" s="6" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="B2" s="7">
         <v>77.54</v>
@@ -12919,7 +12997,7 @@
         <v>87.5</v>
       </c>
       <c r="X2" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Y2" s="11">
         <f>X2*(1+AA2)</f>
@@ -12936,7 +13014,7 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3" s="8" t="s">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="B3" s="7">
         <v>72</v>
@@ -13009,10 +13087,10 @@
         <v>84.88</v>
       </c>
       <c r="X3" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Y3" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Z3">
         <f t="shared" ref="Z3:Z32" si="0">((V3-U3)/U3+(W3-V3)/V3)/2</f>
@@ -13025,7 +13103,7 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4" s="6" t="s">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="B4" s="7">
         <v>26.09</v>
@@ -13094,10 +13172,10 @@
         <v>61.14</v>
       </c>
       <c r="X4" s="7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="Y4" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="Z4">
         <f t="shared" si="0"/>
@@ -13110,7 +13188,7 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5" s="8" t="s">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="B5" s="7">
         <v>34.9</v>
@@ -13183,10 +13261,10 @@
         <v>63.42</v>
       </c>
       <c r="X5" s="7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Y5" s="7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="Z5">
         <f t="shared" si="0"/>
@@ -13268,10 +13346,10 @@
         <v>68.21</v>
       </c>
       <c r="X6" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="Z6">
         <f t="shared" si="0"/>
@@ -13284,7 +13362,7 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7" s="6" t="s">
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="B7" s="7">
         <v>54.24</v>
@@ -13371,7 +13449,7 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8" s="6" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="B8" s="7">
         <v>49.66</v>
@@ -13440,7 +13518,7 @@
         <v>63.36</v>
       </c>
       <c r="X8" s="7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="Y8" s="11">
         <f t="shared" si="2"/>
@@ -13457,7 +13535,7 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9" s="6" t="s">
-        <v>11</v>
+        <v>72</v>
       </c>
       <c r="B9" s="7">
         <v>51.94</v>
@@ -13526,7 +13604,7 @@
         <v>65.69</v>
       </c>
       <c r="X9" s="7" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="Y9" s="11">
         <f t="shared" si="2"/>
@@ -13543,7 +13621,7 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10" s="6" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="B10" s="7">
         <v>88.31</v>
@@ -13634,7 +13712,7 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11" s="6" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="B11" s="7">
         <v>41.5</v>
@@ -13703,10 +13781,10 @@
         <v>73.94</v>
       </c>
       <c r="X11" s="7" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="Y11" s="7" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="Z11">
         <f t="shared" si="0"/>
@@ -13719,7 +13797,7 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12" s="6" t="s">
-        <v>14</v>
+        <v>78</v>
       </c>
       <c r="B12" s="7">
         <v>48.7</v>
@@ -13788,10 +13866,10 @@
         <v>72.66</v>
       </c>
       <c r="X12" s="7" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="Y12" s="7" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="Z12">
         <f t="shared" si="0"/>
@@ -13804,7 +13882,7 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13" s="6" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="B13" s="7">
         <v>28</v>
@@ -13873,10 +13951,10 @@
         <v>59.39</v>
       </c>
       <c r="X13" s="7" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="Y13" s="7" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="Z13">
         <f t="shared" si="0"/>
@@ -13889,7 +13967,7 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="B14" s="7">
         <v>41.96</v>
@@ -13958,10 +14036,10 @@
         <v>69.7</v>
       </c>
       <c r="X14" s="7" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="Z14">
         <f t="shared" si="0"/>
@@ -13974,7 +14052,7 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15" s="6" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="B15" s="7">
         <v>27.69</v>
@@ -14043,7 +14121,7 @@
         <v>61.46</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="Y15" s="11">
         <f t="shared" ref="Y15:Y18" si="3">X15*(1+AA15)</f>
@@ -14060,7 +14138,7 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16" s="8" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="B16" s="7">
         <v>38</v>
@@ -14133,10 +14211,10 @@
         <v>63.94</v>
       </c>
       <c r="X16" s="7" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="Y16" s="7" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="Z16">
         <f t="shared" si="0"/>
@@ -14149,7 +14227,7 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17" s="6" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="B17" s="7">
         <v>23.2</v>
@@ -14218,7 +14296,7 @@
         <v>56.45</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="Y17" s="11">
         <f t="shared" si="3"/>
@@ -14235,7 +14313,7 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18" s="8" t="s">
-        <v>20</v>
+        <v>94</v>
       </c>
       <c r="B18" s="7">
         <v>40.5</v>
@@ -14308,7 +14386,7 @@
         <v>64.09</v>
       </c>
       <c r="X18" s="7" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="Y18" s="11">
         <f t="shared" si="3"/>
@@ -14325,7 +14403,7 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19" s="6" t="s">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="B19" s="7">
         <v>29.75</v>
@@ -14394,10 +14472,10 @@
         <v>59.71</v>
       </c>
       <c r="X19" s="7" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="Y19" s="7" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="Z19">
         <f t="shared" si="0"/>
@@ -14410,7 +14488,7 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20" s="6" t="s">
-        <v>22</v>
+        <v>99</v>
       </c>
       <c r="B20" s="7">
         <v>55</v>
@@ -14483,7 +14561,7 @@
         <v>74.63</v>
       </c>
       <c r="X20" s="7" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="Y20" s="11">
         <f t="shared" ref="Y20:Y28" si="8">X20*(1+AA20)</f>
@@ -14569,7 +14647,7 @@
         <v>55.08</v>
       </c>
       <c r="X21" s="7" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="Y21" s="11">
         <f t="shared" si="8"/>
@@ -14586,7 +14664,7 @@
     </row>
     <row r="22" spans="1:27">
       <c r="A22" s="6" t="s">
-        <v>24</v>
+        <v>102</v>
       </c>
       <c r="B22" s="7">
         <v>40.7</v>
@@ -14659,10 +14737,10 @@
         <v>60.97</v>
       </c>
       <c r="X22" s="7" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="Y22" s="7" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="Z22">
         <f t="shared" si="0"/>
@@ -14675,7 +14753,7 @@
     </row>
     <row r="23" spans="1:27">
       <c r="A23" s="6" t="s">
-        <v>25</v>
+        <v>105</v>
       </c>
       <c r="B23" s="7">
         <v>33.1</v>
@@ -14748,10 +14826,10 @@
         <v>70.32</v>
       </c>
       <c r="X23" s="7" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="Y23" s="7" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="Z23">
         <f t="shared" si="0"/>
@@ -14764,7 +14842,7 @@
     </row>
     <row r="24" spans="1:27">
       <c r="A24" s="6" t="s">
-        <v>26</v>
+        <v>108</v>
       </c>
       <c r="B24" s="7">
         <v>26.7</v>
@@ -14837,10 +14915,10 @@
         <v>57.82</v>
       </c>
       <c r="X24" s="7" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="Y24" s="7" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="Z24">
         <f t="shared" si="0"/>
@@ -14853,7 +14931,7 @@
     </row>
     <row r="25" spans="1:27">
       <c r="A25" s="6" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="B25" s="7">
         <v>23.87</v>
@@ -14922,7 +15000,7 @@
         <v>54.33</v>
       </c>
       <c r="X25" s="7" t="s">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="Y25" s="11">
         <f t="shared" si="8"/>
@@ -14939,7 +15017,7 @@
     </row>
     <row r="26" spans="1:27">
       <c r="A26" s="6" t="s">
-        <v>28</v>
+        <v>113</v>
       </c>
       <c r="B26" s="7">
         <v>23.36</v>
@@ -15008,7 +15086,7 @@
         <v>51.05</v>
       </c>
       <c r="X26" s="7" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="Y26" s="11">
         <f t="shared" si="8"/>
@@ -15094,7 +15172,7 @@
         <v>36.61</v>
       </c>
       <c r="X27" s="7" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="Y27" s="11">
         <f t="shared" si="8"/>
@@ -15111,7 +15189,7 @@
     </row>
     <row r="28" spans="1:27">
       <c r="A28" s="6" t="s">
-        <v>30</v>
+        <v>116</v>
       </c>
       <c r="B28" s="7">
         <v>32.27</v>
@@ -15198,7 +15276,7 @@
     </row>
     <row r="29" spans="1:27">
       <c r="A29" s="6" t="s">
-        <v>31</v>
+        <v>117</v>
       </c>
       <c r="B29" s="7">
         <v>24.41</v>
@@ -15267,10 +15345,10 @@
         <v>53.33</v>
       </c>
       <c r="X29" s="7" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="Y29" s="7" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="Z29">
         <f t="shared" si="0"/>
@@ -15283,7 +15361,7 @@
     </row>
     <row r="30" spans="1:27">
       <c r="A30" s="6" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="B30" s="7">
         <v>34.76</v>
@@ -15352,10 +15430,10 @@
         <v>61.02</v>
       </c>
       <c r="X30" s="7" t="s">
-        <v>95</v>
+        <v>121</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>96</v>
+        <v>122</v>
       </c>
       <c r="Z30">
         <f t="shared" si="0"/>
@@ -15437,7 +15515,7 @@
         <v>66.04</v>
       </c>
       <c r="X31" s="7" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="Y31" s="11">
         <f>X31*(1+AA31)</f>
@@ -15523,7 +15601,7 @@
         <v>57.26</v>
       </c>
       <c r="X32" s="7" t="s">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="Y32" s="11">
         <f>X32*(1+AA32)</f>
@@ -15676,7 +15754,7 @@
         <v>1550</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>99</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -15697,7 +15775,7 @@
         <v>4889</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -15723,7 +15801,7 @@
         <v>31.7038249130702</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>101</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="2:6">
@@ -15735,7 +15813,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -15745,7 +15823,7 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="1" t="s">
-        <v>103</v>
+        <v>129</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -15754,7 +15832,7 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="1" t="s">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -15770,7 +15848,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>

</xml_diff>